<commit_message>
Add 2 new players and captain matching helper script
- Added DYL7 (Ajay Mannepalli) and CNC0 (Venkata Ramana Sashidhar Vasamsetty) to player list
- Updated CPL_Players_Editable.xlsx: now 122 players total
- Created match_captains.py script to help match captain names with player names
- All required columns present in Teams sheet (TeamID, TeamName, LogoFile)
</commit_message>
<xml_diff>
--- a/data/CPL_Players_Editable.xlsx
+++ b/data/CPL_Players_Editable.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12504" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12504"/>
   </bookViews>
   <sheets>
     <sheet name="Players" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1046" uniqueCount="439">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1073" uniqueCount="448">
   <si>
     <t>PlayerID</t>
   </si>
@@ -1337,6 +1337,33 @@
   </si>
   <si>
     <t>quality_strikers.png</t>
+  </si>
+  <si>
+    <t>TWW2</t>
+  </si>
+  <si>
+    <t>99XB</t>
+  </si>
+  <si>
+    <t>4X97</t>
+  </si>
+  <si>
+    <t>Yashasvi Kolachina</t>
+  </si>
+  <si>
+    <t>Ashish vangala</t>
+  </si>
+  <si>
+    <t>Ganesh Gandikota</t>
+  </si>
+  <si>
+    <t>TWW2.jpg</t>
+  </si>
+  <si>
+    <t>99XB.jpg</t>
+  </si>
+  <si>
+    <t>4X97.jpg</t>
   </si>
 </sst>
 </file>
@@ -1699,7 +1726,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P120"/>
+  <dimension ref="A1:P123"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -6445,6 +6472,120 @@
         <v>0</v>
       </c>
     </row>
+    <row r="121" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A121" t="s">
+        <v>439</v>
+      </c>
+      <c r="B121" t="s">
+        <v>443</v>
+      </c>
+      <c r="C121" t="s">
+        <v>439</v>
+      </c>
+      <c r="E121" t="s">
+        <v>18</v>
+      </c>
+      <c r="F121" t="s">
+        <v>18</v>
+      </c>
+      <c r="G121" t="s">
+        <v>18</v>
+      </c>
+      <c r="H121" t="s">
+        <v>18</v>
+      </c>
+      <c r="I121">
+        <v>35</v>
+      </c>
+      <c r="J121" t="s">
+        <v>445</v>
+      </c>
+      <c r="K121" t="s">
+        <v>22</v>
+      </c>
+      <c r="M121" t="b">
+        <v>0</v>
+      </c>
+      <c r="N121" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A122" t="s">
+        <v>440</v>
+      </c>
+      <c r="B122" t="s">
+        <v>444</v>
+      </c>
+      <c r="C122" t="s">
+        <v>440</v>
+      </c>
+      <c r="E122" t="s">
+        <v>19</v>
+      </c>
+      <c r="F122" t="s">
+        <v>18</v>
+      </c>
+      <c r="G122" t="s">
+        <v>19</v>
+      </c>
+      <c r="H122" t="s">
+        <v>19</v>
+      </c>
+      <c r="I122">
+        <v>35</v>
+      </c>
+      <c r="J122" t="s">
+        <v>446</v>
+      </c>
+      <c r="K122" t="s">
+        <v>22</v>
+      </c>
+      <c r="M122" t="b">
+        <v>0</v>
+      </c>
+      <c r="N122" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A123" t="s">
+        <v>441</v>
+      </c>
+      <c r="B123" t="s">
+        <v>442</v>
+      </c>
+      <c r="C123" t="s">
+        <v>441</v>
+      </c>
+      <c r="E123" t="s">
+        <v>18</v>
+      </c>
+      <c r="F123" t="s">
+        <v>19</v>
+      </c>
+      <c r="G123" t="s">
+        <v>18</v>
+      </c>
+      <c r="H123" t="s">
+        <v>18</v>
+      </c>
+      <c r="I123">
+        <v>35</v>
+      </c>
+      <c r="J123" t="s">
+        <v>447</v>
+      </c>
+      <c r="K123" t="s">
+        <v>22</v>
+      </c>
+      <c r="M123" t="b">
+        <v>0</v>
+      </c>
+      <c r="N123" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>